<commit_message>
Add Roots Analysis parenting apps market overview
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YUs4ThZR7vyJGPPKhVC9wX
</commit_message>
<xml_diff>
--- a/research/03_경쟁앱_비교표.xlsx
+++ b/research/03_경쟁앱_비교표.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="경쟁앱 비교" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성 안내" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="시장 개요" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="경쟁앱 비교" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성 안내" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -70,12 +71,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -443,6 +450,221 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>내용</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>출처</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>시장 규모 (2024)</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>약 17억 달러 (USD 1.69B)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Roots Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>시장 규모 (2025)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>약 19.4억 달러 (USD 1.94B)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Roots Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>전망 (2035)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>약 60.2억 달러 (USD 6.02B)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Roots Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>CAGR</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Roots Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>최대 OS 점유</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Android 약 65%</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Roots Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>최대 지역</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>북미 약 37%</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Roots Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>최고 성장 지역</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>아시아·태평양</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Roots Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>유형별 최대 점유</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>베이비 트래커 앱 약 30%</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Roots Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>유형별 최고 성장</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>공동 육아 앱</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Roots Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>원문 URL</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.rootsanalysis.com/reports/parenting-apps-market.html</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>유의</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>검색으로 확인한 공개 요약이며 원문 직접 열람 전. 인용 전 재확인 필요.</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:X9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -871,7 +1093,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add domestic parenting app comparison and AI trend notes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YUs4ThZR7vyJGPPKhVC9wX
</commit_message>
<xml_diff>
--- a/research/03_경쟁앱_비교표.xlsx
+++ b/research/03_경쟁앱_비교표.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="시장 개요" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="경쟁앱 비교" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성 안내" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기능별 추천 앱" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -71,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -85,6 +86,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -450,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -653,6 +655,40 @@
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>주요 16개 육아 앱 평균 MAU 상승</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>약 24%</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>사용자 제공(미검증)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>글로벌 AI 육아·보육 시장 CAGR</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>22.3%</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>사용자 제공(미검증)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -665,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X9"/>
+  <dimension ref="A1:X15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1088,6 +1124,382 @@
       <c r="W9" s="2" t="inlineStr"/>
       <c r="X9" s="2" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>육아 기록</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>베이비타임 (BabyTime)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>수유·성장·이유식·기저귀·수면 기록</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>0~12개월</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>무료+광고/커머스 연계</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>있음(인앱 광고)</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr">
+        <is>
+          <t>국내 1위 기록 앱, 위젯, 부모 간 실시간 동기화, 직관적 UI</t>
+        </is>
+      </c>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="U10" s="2" t="inlineStr"/>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>이유식 기록이 겹침. 우리: 새 재료 반응·도입 재료 기준 추천</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr"/>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>사용자 제공 자료(미검증)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>병원·건강</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>똑닥 (Ddocdoc)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>병원 예약·접수, 영유아 검진·예방접종 관리</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>영유아 전반</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>유료 멤버십(월/연) + 병원 이용료</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>실시간 대기 현황, 확실한 매출원</t>
+        </is>
+      </c>
+      <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>콘텐츠 앱 아님</t>
+        </is>
+      </c>
+      <c r="U11" s="2" t="inlineStr"/>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>직접 경쟁 아님. 부모 타깃 겹침(모집 채널 후보)</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr"/>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>사용자 제공 자료(미검증)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>병원·건강</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>열나요</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>체온 기록, 해열제 용량·간격 가이드, 교차 복용 알람</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>영유아 전반</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>무료+제약사 광고/제휴</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>있음(제휴)</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>밤샘 간호 상황에 특화</t>
+        </is>
+      </c>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr"/>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>직접 경쟁 아님. 의료 면책 방식 참고</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr"/>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>사용자 제공 자료(미검증)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>임신·예비부모</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>280days</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>주수별 성장 체크, 부부 연동 기록</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>임산부·예비 부모</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>프리미엄 결제 + 제휴(태아보험 등)</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr"/>
+      <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr">
+        <is>
+          <t>일러스트 기반 감성 UI</t>
+        </is>
+      </c>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="U13" s="2" t="inlineStr"/>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>직접 경쟁 아님. 월령 타깃 다름</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr"/>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>사용자 제공 자료(미검증)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>콘텐츠·커뮤니티·커머스</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>베이비빌리 (BabyBilly)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>임신·육아 콘텐츠 커뮤니티, 빌리쇼핑</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>예비 부모~영유아</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>커머스 중개·직판 매출</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr">
+        <is>
+          <t>콘텐츠 기반 커머스</t>
+        </is>
+      </c>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr"/>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>커머스 수익 모델 참고</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr"/>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>사용자 제공 자료(미검증)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>육아 기록</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>베이비 트래커 (Baby Tracker)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>수유·성장 기록, 통계 그래프, 좌/우 모유 타이머</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>신생아</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr"/>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>깔끔한 UI, 통계 그래프</t>
+        </is>
+      </c>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="U15" s="2" t="inlineStr"/>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>기록 앱. 직접 경쟁 아님</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr"/>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>사용자 제공 자료(미검증)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1136,4 +1548,176 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>카테고리</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>앱</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>특징</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>수유·성장 기록</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>베이비타임</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>터치 한 번 기록(모유·분유·이유식·기저귀·수면), 공동 양육자 실시간 연동</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>수유·성장 기록</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>베이비 트래커</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>깔끔한 UI, 통계 그래프, 좌/우 모유 타이머</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>병원·건강</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>똑닥</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>실시간 대기 현황, 접수·예약, 영유아 검진·예방접종</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>병원·건강</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>열나요</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>체온·체중별 해열제 용량·간격, 교차 복용 알람</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AI 트렌드</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>울음소리 분석</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>울음소리로 상태 판별(정확도 주장 90%+, 미검증)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AI 트렌드</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AI 육아 상담 챗봇</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>24시간 상담, 이유식 레시피 제안</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AI 트렌드</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>성장 예측·리포트</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>다음 수유 시점 예측, 또래 대비 발달 분석</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AI 트렌드</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>스마트 완구 연동</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>대화형 교구와 앱 연동, 개인화 학습 콘텐츠</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add storybook/nursery-rhyme competitor research
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YUs4ThZR7vyJGPPKhVC9wX
</commit_message>
<xml_diff>
--- a/research/03_경쟁앱_비교표.xlsx
+++ b/research/03_경쟁앱_비교표.xlsx
@@ -701,16 +701,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X15"/>
+  <dimension ref="A1:X14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
@@ -722,12 +722,12 @@
     <col width="16" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="36" customWidth="1" min="19" max="19"/>
+    <col width="30" customWidth="1" min="20" max="20"/>
     <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="40" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
-    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="50" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="45" customHeight="1">
@@ -860,31 +860,87 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>핑크퐁 아기상어 (예시)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
+          <t>핑크퐁플러스 / 아기상어 키즈 월드 / 핑크퐁 TV</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>더핑크퐁컴퍼니</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>동요·동화 영상, 게임, 학습 활동 (캐릭터 IP)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>유아~어린이</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>앱은 무료+앱 내 구입. 핑크퐁플러스는 월 멤버십(요금 미확인)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>멤버십 시 광고·유해 콘텐츠 차단</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>핑크퐁 TV: 다운로드 영상은 오프라인 시청 가능</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>해당 없음(자체 IP, 확인 필요)</t>
+        </is>
+      </c>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
       <c r="R2" s="2" t="inlineStr"/>
-      <c r="S2" s="2" t="inlineStr"/>
-      <c r="T2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>강력한 캐릭터 IP, 풍부한 콘텐츠, 멤버십 모델 보유</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
       <c r="U2" s="2" t="inlineStr"/>
-      <c r="V2" s="2" t="inlineStr"/>
-      <c r="W2" s="2" t="inlineStr"/>
-      <c r="X2" s="2" t="inlineStr"/>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>우리는 광고 없는 무료+월령 맞춤+이유식 통합. 단 IP 인지도 격차가 큼</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 검색 기준</t>
+        </is>
+      </c>
+      <c r="X2" s="2" t="inlineStr">
+        <is>
+          <t>https://fong.kr/pinkfongplus1/ , https://apps.apple.com/kr/app/id1596897739 , https://apps.apple.com/KR/app/id860497608</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -894,184 +950,484 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>베이비버스 (예시)</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
+          <t>베이비버스 (BabyBus)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>BabyBus</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>동요, 만화, 학습 미니게임(앱별 분리 구성)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>유아</t>
+        </is>
+      </c>
       <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>앱별 구독 표시 예: 1개월 6,600원 / 1년 44,000원 / 연속 월 9,000원 / 연속 연 54,000원 (앱마다 상이)</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>일부 앱 광고 포함 표시</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="inlineStr"/>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="inlineStr"/>
-      <c r="T3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>다수 앱 라인업, 학습·게임 중심</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>앱이 분산되어 있고 구독 가격이 앱마다 다름</t>
+        </is>
+      </c>
       <c r="U3" s="2" t="inlineStr"/>
-      <c r="V3" s="2" t="inlineStr"/>
-      <c r="W3" s="2" t="inlineStr"/>
-      <c r="X3" s="2" t="inlineStr"/>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>우리는 동화·동요·이유식을 한 앱에 통합</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 검색 기준</t>
+        </is>
+      </c>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
+          <t>https://apps.apple.com/kr/app/id962605433</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>동영상</t>
+          <t>영상 플랫폼</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>유튜브 키즈 (예시)</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
+          <t>유튜브 키즈 (YouTube Kids)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>어린이용 영상(동요·동화 포함)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>유아~어린이</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>무료(Premium 등 유료 옵션은 확인 필요)</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>확인 필요(공식 정책 직접 확인)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>타이머 있음(시간 종료 시 앱 잠김)</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>연령대 설정</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>해당 없음</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>보호자 암호로 설정 변경</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="inlineStr"/>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="inlineStr"/>
-      <c r="S4" s="2" t="inlineStr"/>
-      <c r="T4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>보호자 설정(타이머, 검색 제한, 영상·채널 차단, 승인된 콘텐츠 모드), 방대한 콘텐츠</t>
+        </is>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>품질·적합성 통제 한계, 콘텐츠 편차(확인 필요)</t>
+        </is>
+      </c>
       <c r="U4" s="2" t="inlineStr"/>
-      <c r="V4" s="2" t="inlineStr"/>
-      <c r="W4" s="2" t="inlineStr"/>
-      <c r="X4" s="2" t="inlineStr"/>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>우리는 사람 검수를 거친 큐레이션 콘텐츠만 제공</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 검색 기준</t>
+        </is>
+      </c>
+      <c r="X4" s="2" t="inlineStr">
+        <is>
+          <t>https://apps.apple.com/KR/app/id936971630 , https://www.inews24.com/view/1023419</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>동화/전자책</t>
+          <t>동요·동화 오디오</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>(전집·전자책 앱 1)</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
+          <t>코코지 (COCOJI)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>동요·동화 오디오(핑크퐁, 베베핀, 뽀로로, 엄마까투리, 로보카폴리 등 제공 소개)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>유아</t>
+        </is>
+      </c>
       <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>구독 서비스 '코코지 올데이' 있음(가격 미확인)</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>해당 없음</t>
+        </is>
+      </c>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="inlineStr"/>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="inlineStr"/>
-      <c r="S5" s="2" t="inlineStr"/>
-      <c r="T5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>여러 인기 IP를 한 앱에 모음</t>
+        </is>
+      </c>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
       <c r="U5" s="2" t="inlineStr"/>
-      <c r="V5" s="2" t="inlineStr"/>
-      <c r="W5" s="2" t="inlineStr"/>
-      <c r="X5" s="2" t="inlineStr"/>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>가장 유사한 통합 모델. 우리는 이유식·잠자리 모드·광고 없음으로 차별화</t>
+        </is>
+      </c>
+      <c r="W5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 검색 기준</t>
+        </is>
+      </c>
+      <c r="X5" s="2" t="inlineStr">
+        <is>
+          <t>https://apps.apple.com/us/app/id1581056078</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>동요/음원</t>
+          <t>동요·학습</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>(동요 음원 앱 1)</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
+          <t>KidloLand (키들로랜드)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>KidloLand</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>동요·이야기·게임 3,000개 이상</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2세 이상</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>앱 내 구입(번들 구독 추정, 가격 미확인)</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr"/>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
       <c r="R6" s="2" t="inlineStr"/>
-      <c r="S6" s="2" t="inlineStr"/>
-      <c r="T6" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>대량 콘텐츠, 번들</t>
+        </is>
+      </c>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>해외 앱, 한국어·한국 정서 적합성 확인 필요</t>
+        </is>
+      </c>
       <c r="U6" s="2" t="inlineStr"/>
-      <c r="V6" s="2" t="inlineStr"/>
-      <c r="W6" s="2" t="inlineStr"/>
-      <c r="X6" s="2" t="inlineStr"/>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>우리는 한국어·월령 맞춤</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 검색 기준</t>
+        </is>
+      </c>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t>https://apps.apple.com/kr/app-bundle/id1653964084</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>이유식 레시피</t>
+          <t>동화</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>(이유식 레시피 앱 1)</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
+          <t>앱스토어 동화 앱 일반 (개별 앱명 추가 확인 필요)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>동화 컬렉션, 일러스트·애니메이션, 음성 내레이션, 부모 목소리 녹음, 자장가 모드</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>2~8세(앱별)</t>
+        </is>
+      </c>
       <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>무료+앱 내 구입 표시</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>자장가 모드 소개 앱 있음(우리 잠자리 모드와 유사)</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="inlineStr"/>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
       <c r="R7" s="2" t="inlineStr"/>
-      <c r="S7" s="2" t="inlineStr"/>
-      <c r="T7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>부모 녹음, 자장가 모드 등 우리 핵심 기능과 겹침</t>
+        </is>
+      </c>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
       <c r="U7" s="2" t="inlineStr"/>
-      <c r="V7" s="2" t="inlineStr"/>
-      <c r="W7" s="2" t="inlineStr"/>
-      <c r="X7" s="2" t="inlineStr"/>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>잠자리 모드와 부모 녹음류 기능은 차별점이 되기 어려울 수 있음. 타이머·볼륨 감소·월령 연계로 차별화 검토</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 검색 기준</t>
+        </is>
+      </c>
+      <c r="X7" s="2" t="inlineStr">
+        <is>
+          <t>https://apps.apple.com/kr/app/id486365921 , https://apps.apple.com/KR/app/id947235578</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>육아 기록</t>
+          <t>동요(구형)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>(육아 기록 앱 1)</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
+          <t>뽀로로 동요놀이</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>LG유플러스·아이코닉스</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>동요 놀이</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>유아</t>
+        </is>
+      </c>
       <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr"/>
@@ -1083,107 +1439,155 @@
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
       <c r="R8" s="2" t="inlineStr"/>
-      <c r="S8" s="2" t="inlineStr"/>
-      <c r="T8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="inlineStr">
+        <is>
+          <t>뽀로로 IP</t>
+        </is>
+      </c>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>2018년 출시 기사 기준, 현재 운영 여부 불명</t>
+        </is>
+      </c>
       <c r="U8" s="2" t="inlineStr"/>
-      <c r="V8" s="2" t="inlineStr"/>
-      <c r="W8" s="2" t="inlineStr"/>
-      <c r="X8" s="2" t="inlineStr"/>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>참고용. 현재 운영 확인 후 유지/삭제</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 검색 기준</t>
+        </is>
+      </c>
+      <c r="X8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gamemeca.com/view.php?gid=114312</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>통합형</t>
+          <t>육아 기록</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>(동화+동요+이유식 통합 앱, 있다면)</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
-      <c r="N9" s="2" t="inlineStr"/>
-      <c r="O9" s="2" t="inlineStr"/>
-      <c r="P9" s="2" t="inlineStr"/>
-      <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="inlineStr"/>
-      <c r="S9" s="2" t="inlineStr"/>
-      <c r="T9" s="2" t="inlineStr"/>
-      <c r="U9" s="2" t="inlineStr"/>
-      <c r="V9" s="2" t="inlineStr"/>
-      <c r="W9" s="2" t="inlineStr"/>
-      <c r="X9" s="2" t="inlineStr"/>
+          <t>베이비타임 (BabyTime)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>수유·성장·이유식·기저귀·수면 기록</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>0~12개월</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>무료+광고/커머스 연계</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>있음(인앱 광고)</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="n"/>
+      <c r="M9" s="2" t="n"/>
+      <c r="N9" s="2" t="n"/>
+      <c r="O9" s="2" t="n"/>
+      <c r="P9" s="2" t="n"/>
+      <c r="Q9" s="2" t="n"/>
+      <c r="R9" s="2" t="n"/>
+      <c r="S9" s="2" t="inlineStr">
+        <is>
+          <t>국내 1위 기록 앱, 위젯, 부모 간 실시간 동기화, 직관적 UI</t>
+        </is>
+      </c>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="n"/>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>이유식 기록이 겹침. 우리: 새 재료 반응·도입 재료 기준 추천</t>
+        </is>
+      </c>
+      <c r="W9" s="2" t="n"/>
+      <c r="X9" s="2" t="inlineStr">
+        <is>
+          <t>사용자 제공 자료(미검증)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>육아 기록</t>
+          <t>병원·건강</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>베이비타임 (BabyTime)</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr"/>
+          <t>똑닥 (Ddocdoc)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>수유·성장·이유식·기저귀·수면 기록</t>
+          <t>병원 예약·접수, 영유아 검진·예방접종 관리</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>0~12개월</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr"/>
+          <t>영유아 전반</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>무료+광고/커머스 연계</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>있음(인앱 광고)</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr"/>
-      <c r="N10" s="2" t="inlineStr"/>
-      <c r="O10" s="2" t="inlineStr"/>
-      <c r="P10" s="2" t="inlineStr"/>
-      <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr"/>
+          <t>유료 멤버십(월/연) + 병원 이용료</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="n"/>
+      <c r="K10" s="2" t="n"/>
+      <c r="L10" s="2" t="n"/>
+      <c r="M10" s="2" t="n"/>
+      <c r="N10" s="2" t="n"/>
+      <c r="O10" s="2" t="n"/>
+      <c r="P10" s="2" t="n"/>
+      <c r="Q10" s="2" t="n"/>
+      <c r="R10" s="2" t="n"/>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>국내 1위 기록 앱, 위젯, 부모 간 실시간 동기화, 직관적 UI</t>
+          <t>실시간 대기 현황, 확실한 매출원</t>
         </is>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>(확인 필요)</t>
-        </is>
-      </c>
-      <c r="U10" s="2" t="inlineStr"/>
+          <t>콘텐츠 앱 아님</t>
+        </is>
+      </c>
+      <c r="U10" s="2" t="n"/>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>이유식 기록이 겹침. 우리: 새 재료 반응·도입 재료 기준 추천</t>
-        </is>
-      </c>
-      <c r="W10" s="2" t="inlineStr"/>
+          <t>직접 경쟁 아님. 부모 타깃 겹침(모집 채널 후보)</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="n"/>
       <c r="X10" s="2" t="inlineStr">
         <is>
           <t>사용자 제공 자료(미검증)</t>
@@ -1198,13 +1602,13 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>똑닥 (Ddocdoc)</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr"/>
+          <t>열나요</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n"/>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>병원 예약·접수, 영유아 검진·예방접종 관리</t>
+          <t>체온 기록, 해열제 용량·간격 가이드, 교차 복용 알람</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1212,40 +1616,44 @@
           <t>영유아 전반</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>유료 멤버십(월/연) + 병원 이용료</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" s="2" t="inlineStr"/>
-      <c r="N11" s="2" t="inlineStr"/>
-      <c r="O11" s="2" t="inlineStr"/>
-      <c r="P11" s="2" t="inlineStr"/>
-      <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr"/>
+          <t>무료+제약사 광고/제휴</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>있음(제휴)</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" s="2" t="n"/>
+      <c r="M11" s="2" t="n"/>
+      <c r="N11" s="2" t="n"/>
+      <c r="O11" s="2" t="n"/>
+      <c r="P11" s="2" t="n"/>
+      <c r="Q11" s="2" t="n"/>
+      <c r="R11" s="2" t="n"/>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>실시간 대기 현황, 확실한 매출원</t>
+          <t>밤샘 간호 상황에 특화</t>
         </is>
       </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t>콘텐츠 앱 아님</t>
-        </is>
-      </c>
-      <c r="U11" s="2" t="inlineStr"/>
+          <t>(확인 필요)</t>
+        </is>
+      </c>
+      <c r="U11" s="2" t="n"/>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t>직접 경쟁 아님. 부모 타깃 겹침(모집 채널 후보)</t>
-        </is>
-      </c>
-      <c r="W11" s="2" t="inlineStr"/>
+          <t>직접 경쟁 아님. 의료 면책 방식 참고</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="n"/>
       <c r="X11" s="2" t="inlineStr">
         <is>
           <t>사용자 제공 자료(미검증)</t>
@@ -1255,49 +1663,45 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>병원·건강</t>
+          <t>임신·예비부모</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>열나요</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr"/>
+          <t>280days</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n"/>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>체온 기록, 해열제 용량·간격 가이드, 교차 복용 알람</t>
+          <t>주수별 성장 체크, 부부 연동 기록</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>영유아 전반</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr"/>
+          <t>임산부·예비 부모</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>무료+제약사 광고/제휴</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>있음(제휴)</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="2" t="inlineStr"/>
-      <c r="O12" s="2" t="inlineStr"/>
-      <c r="P12" s="2" t="inlineStr"/>
-      <c r="Q12" s="2" t="inlineStr"/>
-      <c r="R12" s="2" t="inlineStr"/>
+          <t>프리미엄 결제 + 제휴(태아보험 등)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="n"/>
+      <c r="K12" s="2" t="n"/>
+      <c r="L12" s="2" t="n"/>
+      <c r="M12" s="2" t="n"/>
+      <c r="N12" s="2" t="n"/>
+      <c r="O12" s="2" t="n"/>
+      <c r="P12" s="2" t="n"/>
+      <c r="Q12" s="2" t="n"/>
+      <c r="R12" s="2" t="n"/>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>밤샘 간호 상황에 특화</t>
+          <t>일러스트 기반 감성 UI</t>
         </is>
       </c>
       <c r="T12" s="2" t="inlineStr">
@@ -1305,13 +1709,13 @@
           <t>(확인 필요)</t>
         </is>
       </c>
-      <c r="U12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="n"/>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>직접 경쟁 아님. 의료 면책 방식 참고</t>
-        </is>
-      </c>
-      <c r="W12" s="2" t="inlineStr"/>
+          <t>직접 경쟁 아님. 월령 타깃 다름</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="n"/>
       <c r="X12" s="2" t="inlineStr">
         <is>
           <t>사용자 제공 자료(미검증)</t>
@@ -1321,45 +1725,45 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>임신·예비부모</t>
+          <t>콘텐츠·커뮤니티·커머스</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>280days</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr"/>
+          <t>베이비빌리 (BabyBilly)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n"/>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>주수별 성장 체크, 부부 연동 기록</t>
+          <t>임신·육아 콘텐츠 커뮤니티, 빌리쇼핑</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>임산부·예비 부모</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr"/>
+          <t>예비 부모~영유아</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>프리미엄 결제 + 제휴(태아보험 등)</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="inlineStr"/>
-      <c r="N13" s="2" t="inlineStr"/>
-      <c r="O13" s="2" t="inlineStr"/>
-      <c r="P13" s="2" t="inlineStr"/>
-      <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr"/>
+          <t>커머스 중개·직판 매출</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="n"/>
+      <c r="M13" s="2" t="n"/>
+      <c r="N13" s="2" t="n"/>
+      <c r="O13" s="2" t="n"/>
+      <c r="P13" s="2" t="n"/>
+      <c r="Q13" s="2" t="n"/>
+      <c r="R13" s="2" t="n"/>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>일러스트 기반 감성 UI</t>
+          <t>콘텐츠 기반 커머스</t>
         </is>
       </c>
       <c r="T13" s="2" t="inlineStr">
@@ -1367,13 +1771,13 @@
           <t>(확인 필요)</t>
         </is>
       </c>
-      <c r="U13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="n"/>
       <c r="V13" s="2" t="inlineStr">
         <is>
-          <t>직접 경쟁 아님. 월령 타깃 다름</t>
-        </is>
-      </c>
-      <c r="W13" s="2" t="inlineStr"/>
+          <t>커머스 수익 모델 참고</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="n"/>
       <c r="X13" s="2" t="inlineStr">
         <is>
           <t>사용자 제공 자료(미검증)</t>
@@ -1383,45 +1787,41 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>콘텐츠·커뮤니티·커머스</t>
+          <t>육아 기록</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>베이비빌리 (BabyBilly)</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr"/>
+          <t>베이비 트래커 (Baby Tracker)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>임신·육아 콘텐츠 커뮤니티, 빌리쇼핑</t>
+          <t>수유·성장 기록, 통계 그래프, 좌/우 모유 타이머</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>예비 부모~영유아</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>커머스 중개·직판 매출</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
-      <c r="N14" s="2" t="inlineStr"/>
-      <c r="O14" s="2" t="inlineStr"/>
-      <c r="P14" s="2" t="inlineStr"/>
-      <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="inlineStr"/>
+          <t>신생아</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="n"/>
+      <c r="L14" s="2" t="n"/>
+      <c r="M14" s="2" t="n"/>
+      <c r="N14" s="2" t="n"/>
+      <c r="O14" s="2" t="n"/>
+      <c r="P14" s="2" t="n"/>
+      <c r="Q14" s="2" t="n"/>
+      <c r="R14" s="2" t="n"/>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>콘텐츠 기반 커머스</t>
+          <t>깔끔한 UI, 통계 그래프</t>
         </is>
       </c>
       <c r="T14" s="2" t="inlineStr">
@@ -1429,72 +1829,14 @@
           <t>(확인 필요)</t>
         </is>
       </c>
-      <c r="U14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="n"/>
       <c r="V14" s="2" t="inlineStr">
         <is>
-          <t>커머스 수익 모델 참고</t>
-        </is>
-      </c>
-      <c r="W14" s="2" t="inlineStr"/>
+          <t>기록 앱. 직접 경쟁 아님</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="n"/>
       <c r="X14" s="2" t="inlineStr">
-        <is>
-          <t>사용자 제공 자료(미검증)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>육아 기록</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>베이비 트래커 (Baby Tracker)</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>수유·성장 기록, 통계 그래프, 좌/우 모유 타이머</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>신생아</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr"/>
-      <c r="N15" s="2" t="inlineStr"/>
-      <c r="O15" s="2" t="inlineStr"/>
-      <c r="P15" s="2" t="inlineStr"/>
-      <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="inlineStr"/>
-      <c r="S15" s="2" t="inlineStr">
-        <is>
-          <t>깔끔한 UI, 통계 그래프</t>
-        </is>
-      </c>
-      <c r="T15" s="2" t="inlineStr">
-        <is>
-          <t>(확인 필요)</t>
-        </is>
-      </c>
-      <c r="U15" s="2" t="inlineStr"/>
-      <c r="V15" s="2" t="inlineStr">
-        <is>
-          <t>기록 앱. 직접 경쟁 아님</t>
-        </is>
-      </c>
-      <c r="W15" s="2" t="inlineStr"/>
-      <c r="X15" s="2" t="inlineStr">
         <is>
           <t>사용자 제공 자료(미검증)</t>
         </is>

</xml_diff>

<commit_message>
Add RAG personalized story generation and Typecast narration proposal
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YUs4ThZR7vyJGPPKhVC9wX
</commit_message>
<xml_diff>
--- a/research/03_경쟁앱_비교표.xlsx
+++ b/research/03_경쟁앱_비교표.xlsx
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X14"/>
+  <dimension ref="A1:X17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1842,6 +1842,132 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>울음 분석</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>babycryinterpreter.com</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr"/>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr"/>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>울음 분석. 정확도·가격 확인 필요</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr"/>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>멘토링 자료 벤치마킹 대상(내용 미조사)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>이유식 레시피</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>스푼타임</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr"/>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>이유식 레시피. 상세 확인 필요</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr"/>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>멘토링 자료 벤치마킹 대상(내용 미조사)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>육아 기록</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>삐요로그</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr"/>
+      <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr"/>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>기록·생활 패턴 관리. 상세 확인 필요</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr"/>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>멘토링 자료 벤치마킹 대상(내용 미조사)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>